<commit_message>
Adding B2B Booking Test
</commit_message>
<xml_diff>
--- a/TestData/TestData.xlsx
+++ b/TestData/TestData.xlsx
@@ -9,12 +9,13 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8100" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8100"/>
   </bookViews>
   <sheets>
     <sheet name="Consolidator_Login" sheetId="1" r:id="rId1"/>
     <sheet name="C2C_Booking" sheetId="2" r:id="rId2"/>
     <sheet name="Connote_Acceptance" sheetId="3" r:id="rId3"/>
+    <sheet name="B2B_Booking" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="56">
   <si>
     <t>Username</t>
   </si>
@@ -163,7 +164,37 @@
     <t>ShipmentNo</t>
   </si>
   <si>
-    <t>REF-32618</t>
+    <t>Payment Option</t>
+  </si>
+  <si>
+    <t>CASH</t>
+  </si>
+  <si>
+    <t>CustomerName</t>
+  </si>
+  <si>
+    <t>ShipperFirstName</t>
+  </si>
+  <si>
+    <t>ALIBABA [ALIBABA-1246]</t>
+  </si>
+  <si>
+    <t>SHANGHAI SHA BRANCH [CB250000107]</t>
+  </si>
+  <si>
+    <t>ShipperCustomsRegNo</t>
+  </si>
+  <si>
+    <t>SHANGHAI12345</t>
+  </si>
+  <si>
+    <t>ConsigneeCustomsRegNo</t>
+  </si>
+  <si>
+    <t>Addis123456</t>
+  </si>
+  <si>
+    <t>REF-32733</t>
   </si>
 </sst>
 </file>
@@ -558,7 +589,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>4</v>
@@ -728,24 +759,236 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.36328125" customWidth="1"/>
+    <col min="2" max="2" width="17.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>44</v>
       </c>
+      <c r="B1" s="7" t="s">
+        <v>45</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>55</v>
+      </c>
+      <c r="B2" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AD2"/>
+  <sheetFormatPr defaultColWidth="17.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.90625" customWidth="1"/>
+    <col min="2" max="2" width="34.6328125" customWidth="1"/>
+    <col min="11" max="11" width="20.81640625" customWidth="1"/>
+    <col min="21" max="21" width="22.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:30" ht="29" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD1" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="5">
+        <v>91</v>
+      </c>
+      <c r="J2" s="5">
+        <v>4875643323</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="O2" s="5">
+        <v>1000</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="S2" s="5">
+        <v>91</v>
+      </c>
+      <c r="T2" s="5">
+        <v>5647647453</v>
+      </c>
+      <c r="U2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="W2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y2" s="5">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="5">
+        <v>10</v>
+      </c>
+      <c r="AA2" s="5">
+        <v>10</v>
+      </c>
+      <c r="AB2" s="5">
+        <v>10</v>
+      </c>
+      <c r="AC2" s="5">
+        <v>10</v>
+      </c>
+      <c r="AD2" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" display="mailto:manish@gmail.com"/>
+    <hyperlink ref="Q2" r:id="rId2" display="mailto:manish.addis@gmail.com"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
+</worksheet>
 </file>
</xml_diff>